<commit_message>
Phase 1 stage 3: detailed design (7 units)
Decompose SWA-001's 7 components into 7 Python units (UNIT-001~007)
with fully specified pseudocode, function contracts, a policy
decision table encoding the Crash>SensorFault>ApproachRisk>Default
priority chain, and a stateless-per-cycle SystemState design that
resolves SWA-001's "recovery condition unspecified" open item at the
mechanism level (still flagged for OEM confirmation). Fill SWD-001
(all 15 template sections), SWD-002 (unit class/call diagram), and
update TRC-001's Detailed Design column.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/traceability/TRC-001_양방향 요구사항 추적 매트릭스.xlsx
+++ b/traceability/TRC-001_양방향 요구사항 추적 매트릭스.xlsx
@@ -797,7 +797,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>UNIT-003 CrashReleaseHandler.tryHandle</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -822,7 +822,7 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>요구사항+아키텍처 할당 완료(Phase1)</t>
+          <t>요구사항+아키텍처+상세설계 할당 완료(Phase1)</t>
         </is>
       </c>
     </row>
@@ -844,7 +844,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>UNIT-003 CrashReleaseHandler.tryHandle</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -869,7 +869,7 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>요구사항+아키텍처 할당 완료(Phase1)</t>
+          <t>요구사항+아키텍처+상세설계 할당 완료(Phase1)</t>
         </is>
       </c>
     </row>
@@ -891,7 +891,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>UNIT-005 ApproachRiskHandler.tryHandle</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -916,7 +916,7 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>요구사항+아키텍처 할당 완료(Phase1)</t>
+          <t>요구사항+아키텍처+상세설계 할당 완료(Phase1)</t>
         </is>
       </c>
     </row>
@@ -938,7 +938,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>UNIT-005 ApproachRiskHandler.tryHandle</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -963,7 +963,7 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>요구사항+아키텍처 할당 완료(Phase1)</t>
+          <t>요구사항+아키텍처+상세설계 할당 완료(Phase1)</t>
         </is>
       </c>
     </row>
@@ -985,7 +985,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>UNIT-005 ApproachRiskHandler.tryHandle</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -1010,7 +1010,7 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>요구사항+아키텍처 할당 완료(Phase1)</t>
+          <t>요구사항+아키텍처+상세설계 할당 완료(Phase1)</t>
         </is>
       </c>
     </row>
@@ -1032,7 +1032,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>UNIT-001 InputValidator.getValidatedSignal</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -1057,7 +1057,7 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>요구사항+아키텍처 할당 완료(Phase1)</t>
+          <t>요구사항+아키텍처+상세설계 할당 완료(Phase1)</t>
         </is>
       </c>
     </row>
@@ -1079,7 +1079,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>UNIT-001 InputValidator.getValidatedSignal</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -1104,7 +1104,7 @@
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>요구사항+아키텍처 할당 완료(Phase1)</t>
+          <t>요구사항+아키텍처+상세설계 할당 완료(Phase1)</t>
         </is>
       </c>
     </row>
@@ -1126,7 +1126,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>UNIT-004 SensorFaultHandler.tryHandle</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -1151,7 +1151,7 @@
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>요구사항+아키텍처 할당 완료(Phase1)</t>
+          <t>요구사항+아키텍처+상세설계 할당 완료(Phase1)</t>
         </is>
       </c>
     </row>
@@ -1173,7 +1173,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>UNIT-004 SensorFaultHandler.tryHandle</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -1198,7 +1198,7 @@
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>요구사항+아키텍처 할당 완료(Phase1)</t>
+          <t>요구사항+아키텍처+상세설계 할당 완료(Phase1)</t>
         </is>
       </c>
     </row>
@@ -1276,7 +1276,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F12"/>
+  <dimension ref="A1:F13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1482,6 +1482,38 @@
         </is>
       </c>
       <c r="F12" t="inlineStr">
+        <is>
+          <t>미승인</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>0.3</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>detailed-designer(AI)</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Phase 1 상세설계(7개 유닛) 할당 반영 — Detailed Design 열 갱신</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>사용자 검토 대기</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
         <is>
           <t>미승인</t>
         </is>

</xml_diff>

<commit_message>
Phase 1 stage 6: system test (9 cases, requirement coverage 100%)
SWR-005,006,007,008,009,013a,013b,021a,021b 9개 항목을 SWR-001 §4.2
수용기준 원문 기준으로 블랙박스 시스템 테스트(VER-CASE-001~009)로 검증.
ChildlockSystem 블랙박스 진입점을 tests/support의 공용 배선(RealChildlockWiring)
위에 얹어 tests/integration과의 중복 배선 코드를 제거(pylint duplicate-code 위반 해소).

- VER-001/VER-002 검증 명세서·결과서 작성, TRC-001 SWE.6 열 갱신
- 51/51 테스트 통과, Branch 커버리지 100%, naming/complexity/duplicate-code 10.00/10
- CI PYTHONPATH를 src:.로 확장(tests.support 공용 픽스처 import 지원)

Phase 1(안전 핵심 로직, ASIL B) 6단계 전체 완료:
요구사항분석 -> 아키텍처설계 -> 상세설계 -> 구현 -> 통합시험 -> 시스템테스트

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/traceability/TRC-001_양방향 요구사항 추적 매트릭스.xlsx
+++ b/traceability/TRC-001_양방향 요구사항 추적 매트릭스.xlsx
@@ -864,12 +864,12 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>VER-CASE-002</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>단위+통합 시험 완료(Phase1), Branch/함수/Call 커버리지 100%(pragma로 방어코드 3라인 제외)</t>
+          <t>단위+통합+시스템 시험 완료(Phase1), Branch/함수/Call 커버리지 100%(pragma로 방어코드 3라인 제외), 요구사항 커버리지 100%, 전체 테스트 성공률 100%</t>
         </is>
       </c>
     </row>
@@ -911,12 +911,12 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>VER-CASE-003</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>단위+통합 시험 완료(Phase1), Branch/함수/Call 커버리지 100%(pragma로 방어코드 3라인 제외)</t>
+          <t>단위+통합+시스템 시험 완료(Phase1), Branch/함수/Call 커버리지 100%(pragma로 방어코드 3라인 제외), 요구사항 커버리지 100%, 전체 테스트 성공률 100%</t>
         </is>
       </c>
     </row>
@@ -958,12 +958,12 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>VER-CASE-004</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>단위+통합 시험 완료(Phase1), Branch/함수/Call 커버리지 100%(pragma로 방어코드 3라인 제외)</t>
+          <t>단위+통합+시스템 시험 완료(Phase1), Branch/함수/Call 커버리지 100%(pragma로 방어코드 3라인 제외), 요구사항 커버리지 100%, 전체 테스트 성공률 100%</t>
         </is>
       </c>
     </row>
@@ -1005,12 +1005,12 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>VER-CASE-005</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>단위+통합 시험 완료(Phase1), Branch/함수/Call 커버리지 100%(pragma로 방어코드 3라인 제외)</t>
+          <t>단위+통합+시스템 시험 완료(Phase1), Branch/함수/Call 커버리지 100%(pragma로 방어코드 3라인 제외), 요구사항 커버리지 100%, 전체 테스트 성공률 100%</t>
         </is>
       </c>
     </row>
@@ -1052,12 +1052,12 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>VER-CASE-006</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>단위+통합 시험 완료(Phase1), Branch/함수/Call 커버리지 100%(pragma로 방어코드 3라인 제외)</t>
+          <t>단위+통합+시스템 시험 완료(Phase1), Branch/함수/Call 커버리지 100%(pragma로 방어코드 3라인 제외), 요구사항 커버리지 100%, 전체 테스트 성공률 100%</t>
         </is>
       </c>
     </row>
@@ -1099,12 +1099,12 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>VER-CASE-007</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>단위+통합 시험 완료(Phase1), Branch/함수/Call 커버리지 100%(pragma로 방어코드 3라인 제외)</t>
+          <t>단위+통합+시스템 시험 완료(Phase1), Branch/함수/Call 커버리지 100%(pragma로 방어코드 3라인 제외), 요구사항 커버리지 100%, 전체 테스트 성공률 100%</t>
         </is>
       </c>
     </row>
@@ -1146,12 +1146,12 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>VER-CASE-008</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>단위+통합 시험 완료(Phase1), Branch/함수/Call 커버리지 100%(pragma로 방어코드 3라인 제외)</t>
+          <t>단위+통합+시스템 시험 완료(Phase1), Branch/함수/Call 커버리지 100%(pragma로 방어코드 3라인 제외), 요구사항 커버리지 100%, 전체 테스트 성공률 100%</t>
         </is>
       </c>
     </row>
@@ -1193,12 +1193,12 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>VER-CASE-009</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>단위+통합 시험 완료(Phase1), Branch/함수/Call 커버리지 100%(pragma로 방어코드 3라인 제외)</t>
+          <t>단위+통합+시스템 시험 완료(Phase1), Branch/함수/Call 커버리지 100%(pragma로 방어코드 3라인 제외), 요구사항 커버리지 100%, 전체 테스트 성공률 100%</t>
         </is>
       </c>
     </row>
@@ -1276,7 +1276,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F15"/>
+  <dimension ref="A1:F37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1578,6 +1578,38 @@
         </is>
       </c>
       <c r="F15" t="inlineStr">
+        <is>
+          <t>미승인</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>0.6</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>sw-system-tester(AI)</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>Phase 1 시스템 테스트(9 케이스) 완료 — SWE.6 열 갱신, 요구사항 커버리지 100%</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>사용자 검토 대기</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
         <is>
           <t>미승인</t>
         </is>

</xml_diff>